<commit_message>
thêm trường số ghê
</commit_message>
<xml_diff>
--- a/static/templates/template_khach_moi.xlsx
+++ b/static/templates/template_khach_moi.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -458,7 +458,8 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,6 +500,11 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Số ghế</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Ghi chú</t>
         </is>
       </c>
@@ -539,6 +545,11 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>Khách VIP</t>
         </is>
       </c>
@@ -577,7 +588,12 @@
           <t>Trưởng phòng</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -615,6 +631,11 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>B01</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Khách mới</t>
         </is>
       </c>
@@ -636,7 +657,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2. Cột 'Họ và tên' và 'Số điện thoại' là bắt buộc</t>
+          <t>2. Cột 'Họ và tên', 'Số điện thoại' và 'Số ghế' là bắt buộc</t>
         </is>
       </c>
     </row>
@@ -650,27 +671,34 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>4. Các cột khác có thể để trống</t>
+          <t>4. Cột 'Số ghế' nhập theo format: A01, B05, C12...</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>5. Lưu file và upload lên hệ thống</t>
+          <t>5. Các cột khác có thể để trống</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>6. Ảnh sẽ được cập nhật sau khi import xong</t>
+          <t>6. Lưu file và upload lên hệ thống</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>7. Ảnh sẽ được cập nhật sau khi import xong</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A6:I6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>